<commit_message>
Poursuite du dev sur les calculs de dilution, correction mineure dans le script de paramétrage (renommage des colonnes)
</commit_message>
<xml_diff>
--- a/02_data/SITOUREF/BET-023-2026_002_Info_points_rejet.xlsx
+++ b/02_data/SITOUREF/BET-023-2026_002_Info_points_rejet.xlsx
@@ -80506,9 +80506,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="3" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="633c736c1f52b59bab6ff2ec826f3b7e">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a8c24be4bccf061f1609b4dbaef8d8d2" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3aafe4bc97fbec4e49b652d28c2caa88">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" xmlns:ns3="a7b14cff-5e05-4f6c-b214-44a9052046af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e93d2fa6853c901024a85aa72cf9a7fe" ns2:_="" ns3:_="">
     <xsd:import namespace="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
+    <xsd:import namespace="a7b14cff-5e05-4f6c-b214-44a9052046af"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -80518,6 +80519,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -80543,6 +80549,43 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2498e138-10ad-4e45-a616-48606944e53a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a7b14cff-5e05-4f6c-b214-44a9052046af" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{e533d34c-d265-4360-97e9-dc06e3d45d14}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a7b14cff-5e05-4f6c-b214-44a9052046af">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
     <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
@@ -80553,8 +80596,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -80654,12 +80697,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="a7b14cff-5e05-4f6c-b214-44a9052046af" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4222387a-a7c4-4a56-bf01-5dca1ac56634">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E478AEA8-CEF0-4E27-BCF5-C3477E330DCF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C69A745-0BFF-47F3-AEAA-ADB216146325}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>